<commit_message>
Add Notebook 06 for benchmarking CVRP against MS6 + TSP
- Introduced a new notebook to compare the performance of the global CVRP solution with the MS6 + TSP approach.
- Implemented data retrieval for students and constructed a distance matrix using OSRM.
- Defined two approaches: one using MS6 + TSP and another using global CVRP.
- Added metrics for measuring performance, including duration, distance, and bus utilization.
- Included visualizations for results and charge balancing across buses.
- Documented the findings and conclusions based on the benchmark results.
</commit_message>
<xml_diff>
--- a/docs/Planning_PFE_Transport_Scolaire.xlsx
+++ b/docs/Planning_PFE_Transport_Scolaire.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="88">
   <si>
     <t>SUIVI D'AVANCEMENT HEBDOMADAIRE — PFE TRANSPORT SCOLAIRE</t>
   </si>
@@ -245,6 +245,120 @@
 Slides soutenance
 Vidéo démo
 Répétition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS6 refonte v3 (data-science) :
+• projection UTM 30N (pyproj) au lieu de StandardScaler → distances vraies en mètres
+• k-médoïdes CAPACITAIRE sur distance ROUTIÈRE OSRM (repli euclidien)
+• affectation globale par programmation linéaire → taille ≤ capacité garantie
+• nombre de bus choisi par courbe de PARETO (qualité vs flotte)
+• 3 notebooks CRISP-DM + benchmark de 11 algorithmes
+Triggers RabbitMQ opérationnels · données v2 (300 élèves Meknès)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart au plan assumé : K-Means/DBSCAN seuls produisaient des groupes INFAISABLES (capacité des bus dépassée). Silhouette 0,43 &lt; 0,5 = arbitrage capacité ↔ compacité, documenté et défendu plutôt que masqué.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 5 déclencheurs de recalcul du clustering (eleve.created / gps.updated / deleted + bus.created / deleted) avec asyncio.Lock anti-rafale
+• Garde-fou qualité DYNAMIQUE : verdict OK / DEGRADE / CRITIQUE, baseline roulante
+• MS12 : dataset 180 jours ancré sur routes OSRM réelles + facteurs marocains (Ramadan, jour de souk, météo, trafic) ; incidents en queue lourde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le garde-fou est INFORMATIF, pas un déclencheur : un seuil fixe à 0,5 serait toujours rouge puisque notre silhouette de conception vaut 0,43. Plancher ancré sur ce point de conception (0,325).
+État de l'art du mémoire NON commencé.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• MS12 : benchmark multi-modèles (baselines → linéaires → forêts → boosting), split TEMPOREL, double vue (tous trajets / trajets normaux)
+  → ElasticNet gagnant : R² 0,82 · MAE 0,86 min · +52,7 % vs baseline OSRM brute
+• Endpoints FastAPI ETA (:8088) + artefact gelé
+• MS9 : agent tool-calling, outils MS1/MS2/MS3/MS10/MS12 scopés au parent par le JWT, reverse geocoding OSM, FR / arabe / darija</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deux écarts au plan, tous deux MESURÉS et non subis :
+1) XGBoost a bien été benchmarké mais ElasticNet l'emporte — le résultat est conservé tel quel plutôt que d'imposer le modèle prévu.
+2) LangChain écarté au profit d'un agent maison (plus simple à auditer et à expliquer) ; Mistral remplacé par gpt-oss/Gemini, Groq ayant décommissionné toute la famille Llama.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• MS9 : pré-fetch des enfants + injection de contexte au prompt, appels d'outils en parallèle, cascade de providers avec retry/backoff
+• MS5 VRP : un TSP par bus (OR-Tools), dépôt = école, coût d'arc = durée routière OSRM réelle → gain +12,6 % vs plus-proche-voisin
+• App mobile PARENT Flutter v1 (Chrome :5174 / Android)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Choix « soir = même ordre que le matin » PROUVÉ par la mesure (verify_sens.py) : l'ordre inversé n'est pas ré-optimisé et coûte ~2× sur matrice OSRM asymétrique ; garder le même ordre équilibre le temps à bord sur la journée.
+/tournees parallélisé (asyncio.gather + OR-Tools en thread) : 43 s → 9 s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Console web React/Vite/TS à 3 rôles (admin · chauffeur · parent) :
+• dashboard KPIs + graphiques, carte live (bus interpolés, ETA, anomalies)
+• clustering : Pareto, diagnostics, cartes de clusters + prévisualisation
+• CRUD élèves/bus/utilisateurs + liaisons parent↔enfant et chauffeur↔bus
+• messagerie chauffeur ↔ admin, diffusion aux parents
+• déviation d'itinéraire (UC-8) : tournée figée au démarrage, surveillée par MS11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Términé partiellement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRP benchmark PARTIEL : seule la baseline plus-proche-voisin a été comparée ; le CVRP global (affectation + routage résolus ensemble) restait à mesurer.
+RÉAFFECTATION DYNAMIQUE (UC-9) NON RÉALISÉE — seul cas d'usage du CDC sans implémentation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• MS11 : dataset propre à anomalies HÉTÉROGÈNES (franc / contextuel / surcharge), feature « surprise » = ratio ajusté au contexte
+• 4 détecteurs comparés à budget d'alerte constant → Isolation Forest CURÉ : PR-AUC 0,91 (vs 0,48 pour la variante diluée), rappel 0,88
+• Monitor GPS live (arrêt prolongé, vitesse excessive) + KPIs dashboard
+• Assistant LLM intégré à l'app Flutter parent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Triple enseignement data-science documenté : (1) le feature engineering prime — « surprise » bat le ratio brut ; (2) la curation prime — iforest curé ≫ dilué ; (3) ici le MULTIVARIÉ gagne, car les anomalies sont hétérogènes.
+Contraste assumé avec MS12, où le modèle SIMPLE l'emporte : c'est le benchmark qui tranche, pas une préférence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Tests end-to-end : e2e_integration_test.py 8/8 (clustering → busId → GPS → ETA → notification → présence → anomalie)
+• Newman (Postman CLI) : 88/88 assertions
+• Documentation GitHub : README, 12 documents techniques dans docs/, CLAUDE.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Términé partiellement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÉPLOIEMENT NON RÉALISÉ : aucun Dockerfile pour les 7 services Java (seuls les 5 services Python en ont), docker-compose limité à l'infrastructure (PostgreSQL/Redis/RabbitMQ/pgAdmin), 15 URLs « localhost » en dur dans la Gateway. Prérequis à lever avant toute mise en ligne Railway/Render.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ETA « le long de la tournée » corrigé sur 5 écrans : distance restante mesurée SUR la polyligne (le point-à-point augmentait pendant le ramassage)
+• Garde anti-extrapolation MS12 : hors du domaine d'entraînement (tronçons 0,7-4 km), bascule sur un facteur de contexte au lieu d'extrapoler
+• Page « Prévisions » parent (web + mobile), endpoint MS5 scopé par le JWT
+• Migration LLM forcée (Llama décommissionné) + refonte de la page de connexion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Términé partiellement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volet technique livré. RÉDACTION DU MÉMOIRE NON COMMENCÉE (chapitres implémentation et résultats).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• App mobile CHAUFFEUR Flutter : 7 écrans, le téléphone devient la SOURCE GPS du bus, file d'écritures hors ligne persistée, 84 tests
+• MS9 Phase B : NL2SQL admin (question → SQL read-only → synthèse)
+• Campagne de correction menée en branchant les apps sur le VRAI backend
+• Benchmark CVRP global vs MS6+TSP (dernière comparaison DS annoncée)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 défauts révélés uniquement par l'exécution sur données réelles :
+1) ETA « cycle fermé » : le compte à rebours bondissait de 1,1 à 35,4 min pile à l'arrivée à l'école (1er et dernier point de la tournée confondus)
+2) MS5 : geometrie et distance_m décrivaient deux trajets (+10,9 % de demi-tours fantômes, faute de continue_straight=false) — polluait aussi la référence MS11
+3) deux crashs d'interface (ListView imbriqué, AnimationController paresseux)
+MÉMOIRE, SLIDES et VIDÉO DÉMO restent à produire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRP benchmark PARTIEL à ce stade : seule la baseline plus-proche-voisin avait été comparée. Le CVRP global (affectation + routage résolus ensemble) a finalement été implémenté et mesuré en S15 — voir la ligne S15.
+RÉAFFECTATION DYNAMIQUE (UC-9) NON RÉALISÉE — seul cas d'usage du CDC sans implémentation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 défauts révélés uniquement par l'exécution sur données réelles :
+1) ETA « cycle fermé » : le compte à rebours bondissait de 1,1 à 35,4 min pile à l'arrivée à l'école (1er et dernier point de la tournée confondus)
+2) MS5 : geometrie et distance_m décrivaient deux trajets (+10,9 % de demi-tours fantômes, faute de continue_straight=false) — polluait aussi la référence MS11
+3) deux crashs d'interface (ListView imbriqué, AnimationController paresseux)
+BENCHMARK CVRP (300 élèves, 7 groupes, budget égalisé) : le CVRP global ne bat JAMAIS la décomposition MS6+TSP de plus de 0,2 %, et lui est le plus souvent inférieur (jusqu'à -2,3 %). Les k-médoïdes de MS6 travaillent déjà sur la distance routière : l'information géographique est injectée AVANT le routage. En revanche le CVRP n'utilise que 6 bus sur 7 (chargés à 50/50) : 1 bus économisé pour +0,4 % de conduite — arbitrage compacité/marge, pas erreur. Verdict mesuré : on garde MS6+TSP.
+MÉMOIRE, SLIDES et VIDÉO DÉMO restent à produire.</t>
   </si>
 </sst>
 </file>
@@ -816,11 +930,15 @@
       <c r="C9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="6"/>
+      <c r="D9" s="6" t="s">
+        <v>65</v>
+      </c>
       <c r="E9" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="6"/>
+        <v>11</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="10" ht="45.0" customHeight="1">
       <c r="A10" s="5" t="s">
@@ -832,11 +950,15 @@
       <c r="C10" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="10"/>
+      <c r="D10" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="11" ht="45.0" customHeight="1">
       <c r="A11" s="5" t="s">
@@ -848,11 +970,15 @@
       <c r="C11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F11" s="6"/>
+      <c r="D11" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="12" ht="45.0" customHeight="1">
       <c r="A12" s="5" t="s">
@@ -864,11 +990,15 @@
       <c r="C12" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F12" s="10"/>
+      <c r="D12" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="13" ht="45.0" customHeight="1">
       <c r="A13" s="5" t="s">
@@ -880,11 +1010,15 @@
       <c r="C13" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F13" s="6"/>
+      <c r="D13" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="14" ht="45.0" customHeight="1">
       <c r="A14" s="5" t="s">
@@ -896,11 +1030,15 @@
       <c r="C14" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="10"/>
-      <c r="E14" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F14" s="10"/>
+      <c r="D14" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="15" ht="45.0" customHeight="1">
       <c r="A15" s="5" t="s">
@@ -912,11 +1050,15 @@
       <c r="C15" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F15" s="6"/>
+      <c r="D15" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="16" ht="45.0" customHeight="1">
       <c r="A16" s="5" t="s">
@@ -928,11 +1070,15 @@
       <c r="C16" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F16" s="10"/>
+      <c r="D16" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="17" ht="45.0" customHeight="1">
       <c r="A17" s="5" t="s">
@@ -944,11 +1090,15 @@
       <c r="C17" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F17" s="6"/>
+      <c r="D17" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1"/>

</xml_diff>